<commit_message>
Pandas | Read Csv & Excel
</commit_message>
<xml_diff>
--- a/top_students.xlsx
+++ b/top_students.xlsx
@@ -413,62 +413,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
           <t>score</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="b">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Execellent</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="b">
-        <v>0</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ahmed</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>95</v>
+      </c>
+      <c r="C3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Execellent</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="b">
-        <v>1</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sara</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>88</v>
+      </c>
+      <c r="C4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Very Good</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>